<commit_message>
Hitos de pago: monto y datos sin negritas; destello en el hito actual
- Datos: el Excel corregido (hito 0 "Inicio de Obra" de COSEGO en
  Picachos; el contrato ya suma 100 %).
- El monto de cada hito y los datos del final (programado, pagado, % del
  contrato) vuelven a texto normal, sin negritas.
- La tarjeta del hito ACTUAL lleva un destello dorado cada 5 s (como los
  prioritarios de Mixtos); sin él con "reducir movimiento" y en el PDF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-cpel/data/HITOS_CARTERA_CPEL.xlsx
+++ b/cartera-cpel/data/HITOS_CARTERA_CPEL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A8D068-AD01-4D85-BE6C-94FB6753284C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD29ECB-E4D7-4B52-A08F-4583220D1099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{80EB7B70-7D9B-4460-9767-FCD518655FC2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{80EB7B70-7D9B-4460-9767-FCD518655FC2}"/>
   </bookViews>
   <sheets>
     <sheet name="PPSIII" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="182">
   <si>
     <t>No.  Hito de Pago y Evento Crítico</t>
   </si>
@@ -632,6 +632,9 @@
   </si>
   <si>
     <t>Fecha programada de pago</t>
+  </si>
+  <si>
+    <t>Inicio de Obra</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1043,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1338,6 +1341,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4632,7 +4647,7 @@
   <sheetPr>
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
@@ -5419,64 +5434,64 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="210" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="27">
-        <v>1</v>
-      </c>
-      <c r="B37" s="61" t="s">
-        <v>148</v>
+        <v>0</v>
+      </c>
+      <c r="B37" s="66" t="s">
+        <v>181</v>
       </c>
       <c r="C37" s="78">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="D37" s="62">
         <v>45523</v>
       </c>
-      <c r="E37" s="79">
+      <c r="E37" s="100">
+        <v>651117.54500000004</v>
+      </c>
+      <c r="F37" s="100"/>
+      <c r="G37" s="101"/>
+      <c r="H37" s="103" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="210" x14ac:dyDescent="0.25">
+      <c r="A38" s="27">
+        <v>1</v>
+      </c>
+      <c r="B38" s="61" t="s">
+        <v>148</v>
+      </c>
+      <c r="C38" s="78">
+        <v>0.05</v>
+      </c>
+      <c r="D38" s="62">
+        <v>45523</v>
+      </c>
+      <c r="E38" s="84">
         <v>162779.39000000001</v>
       </c>
-      <c r="F37" s="80"/>
-      <c r="G37" s="83">
+      <c r="F38" s="80"/>
+      <c r="G38" s="83">
         <v>45838</v>
       </c>
-      <c r="H37" s="81" t="s">
+      <c r="H38" s="102" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="120" x14ac:dyDescent="0.25">
-      <c r="A38" s="86">
+    <row r="39" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A39" s="86">
         <v>2</v>
       </c>
-      <c r="B38" s="63" t="s">
+      <c r="B39" s="63" t="s">
         <v>149</v>
-      </c>
-      <c r="C38" s="12">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="D38" s="24">
-        <v>45586</v>
-      </c>
-      <c r="E38" s="26">
-        <v>244169.08</v>
-      </c>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="A39" s="86">
-        <v>3</v>
-      </c>
-      <c r="B39" s="63" t="s">
-        <v>150</v>
       </c>
       <c r="C39" s="12">
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="D39" s="24">
-        <v>45615</v>
+        <v>45586</v>
       </c>
       <c r="E39" s="26">
         <v>244169.08</v>
@@ -5487,21 +5502,21 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="9">
-        <v>4</v>
+    <row r="40" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A40" s="86">
+        <v>3</v>
       </c>
       <c r="B40" s="63" t="s">
-        <v>151</v>
-      </c>
-      <c r="C40" s="64">
-        <v>0.05</v>
+        <v>150</v>
+      </c>
+      <c r="C40" s="12">
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="D40" s="24">
-        <v>45614</v>
+        <v>45615</v>
       </c>
       <c r="E40" s="26">
-        <v>162779.39000000001</v>
+        <v>244169.08</v>
       </c>
       <c r="F40" s="26"/>
       <c r="G40" s="26"/>
@@ -5509,18 +5524,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" s="63" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C41" s="64">
         <v>0.05</v>
       </c>
       <c r="D41" s="24">
-        <v>45630</v>
+        <v>45614</v>
       </c>
       <c r="E41" s="26">
         <v>162779.39000000001</v>
@@ -5533,19 +5548,19 @@
     </row>
     <row r="42" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A42" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B42" s="63" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C42" s="64">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D42" s="24">
-        <v>45663</v>
+        <v>45630</v>
       </c>
       <c r="E42" s="26">
-        <v>325558.77</v>
+        <v>162779.39000000001</v>
       </c>
       <c r="F42" s="26"/>
       <c r="G42" s="26"/>
@@ -5553,12 +5568,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A43" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43" s="63" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C43" s="64">
         <v>0.1</v>
@@ -5575,18 +5590,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B44" s="63" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C44" s="64">
         <v>0.1</v>
       </c>
       <c r="D44" s="24">
-        <v>45721</v>
+        <v>45663</v>
       </c>
       <c r="E44" s="26">
         <v>325558.77</v>
@@ -5597,18 +5612,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B45" s="63" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C45" s="64">
         <v>0.1</v>
       </c>
       <c r="D45" s="24">
-        <v>45783</v>
+        <v>45721</v>
       </c>
       <c r="E45" s="26">
         <v>325558.77</v>
@@ -5620,132 +5635,130 @@
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="15">
+      <c r="A46" s="9">
+        <v>9</v>
+      </c>
+      <c r="B46" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="C46" s="64">
+        <v>0.1</v>
+      </c>
+      <c r="D46" s="24">
+        <v>45783</v>
+      </c>
+      <c r="E46" s="26">
+        <v>325558.77</v>
+      </c>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="15">
         <v>10</v>
       </c>
-      <c r="B46" s="66" t="s">
+      <c r="B47" s="66" t="s">
         <v>157</v>
       </c>
-      <c r="C46" s="67">
+      <c r="C47" s="67">
         <v>0.1</v>
       </c>
-      <c r="D46" s="20">
+      <c r="D47" s="20">
         <v>45787</v>
       </c>
-      <c r="E46" s="82">
+      <c r="E47" s="82">
         <v>325558.77</v>
       </c>
-      <c r="F46" s="82"/>
-      <c r="G46" s="82"/>
-      <c r="H46" s="11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="27" x14ac:dyDescent="0.25">
-      <c r="A47" s="99" t="s">
+      <c r="F47" s="82"/>
+      <c r="G47" s="82"/>
+      <c r="H47" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="27" x14ac:dyDescent="0.25">
+      <c r="A48" s="99" t="s">
         <v>163</v>
       </c>
-      <c r="B47" s="99"/>
-      <c r="C47" s="99"/>
-      <c r="D47" s="99"/>
-      <c r="E47" s="99"/>
-      <c r="F47" s="99"/>
-      <c r="G47" s="99"/>
-      <c r="H47" s="99"/>
-    </row>
-    <row r="48" spans="1:8" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="77" t="s">
+      <c r="B48" s="99"/>
+      <c r="C48" s="99"/>
+      <c r="D48" s="99"/>
+      <c r="E48" s="99"/>
+      <c r="F48" s="99"/>
+      <c r="G48" s="99"/>
+      <c r="H48" s="99"/>
+    </row>
+    <row r="49" spans="1:8" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="B48" s="77" t="s">
+      <c r="B49" s="77" t="s">
         <v>40</v>
       </c>
-      <c r="C48" s="77" t="s">
+      <c r="C49" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="D48" s="77" t="s">
+      <c r="D49" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="E48" s="77" t="s">
+      <c r="E49" s="77" t="s">
         <v>135</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G48" s="1" t="s">
+      <c r="G49" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H48" s="1" t="s">
+      <c r="H49" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="27">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="27">
         <v>1</v>
       </c>
-      <c r="B49" s="61" t="s">
+      <c r="B50" s="61" t="s">
         <v>158</v>
       </c>
-      <c r="C49" s="78">
+      <c r="C50" s="78">
         <v>0.15</v>
       </c>
-      <c r="D49" s="62">
+      <c r="D50" s="62">
         <v>45397</v>
       </c>
-      <c r="E49" s="79">
+      <c r="E50" s="79">
         <v>6307915.5</v>
       </c>
-      <c r="F49" s="84"/>
-      <c r="G49" s="7">
+      <c r="F50" s="84"/>
+      <c r="G50" s="7">
         <v>45425</v>
       </c>
-      <c r="H49" s="87" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="9">
-        <v>2</v>
-      </c>
-      <c r="B50" s="63" t="s">
-        <v>159</v>
-      </c>
-      <c r="C50" s="64">
-        <v>0.25</v>
-      </c>
-      <c r="D50" s="24">
-        <v>45467</v>
-      </c>
-      <c r="E50" s="26">
-        <v>10513192.49</v>
-      </c>
-      <c r="F50" s="88"/>
-      <c r="G50" s="89">
-        <v>45467</v>
-      </c>
-      <c r="H50" s="81" t="s">
+      <c r="H50" s="87" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B51" s="63" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C51" s="64">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="D51" s="24">
-        <v>45534</v>
+        <v>45467</v>
       </c>
       <c r="E51" s="26">
-        <v>16821107.989999998</v>
+        <v>10513192.49</v>
       </c>
       <c r="F51" s="88"/>
       <c r="G51" s="89">
-        <v>45555</v>
+        <v>45467</v>
       </c>
       <c r="H51" s="81" t="s">
         <v>10</v>
@@ -5753,45 +5766,69 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="9">
+        <v>3</v>
+      </c>
+      <c r="B52" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="C52" s="64">
+        <v>0.4</v>
+      </c>
+      <c r="D52" s="24">
+        <v>45534</v>
+      </c>
+      <c r="E52" s="26">
+        <v>16821107.989999998</v>
+      </c>
+      <c r="F52" s="88"/>
+      <c r="G52" s="89">
+        <v>45555</v>
+      </c>
+      <c r="H52" s="81" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="9">
         <v>4</v>
       </c>
-      <c r="B52" s="63" t="s">
+      <c r="B53" s="63" t="s">
         <v>161</v>
       </c>
-      <c r="C52" s="64">
+      <c r="C53" s="64">
         <v>0.1</v>
       </c>
-      <c r="D52" s="24">
+      <c r="D53" s="24">
         <v>45579</v>
       </c>
-      <c r="E52" s="26">
+      <c r="E53" s="26">
         <v>4205277</v>
       </c>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="15">
+      <c r="F53" s="26"/>
+      <c r="G53" s="26"/>
+      <c r="H53" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="15">
         <v>5</v>
       </c>
-      <c r="B53" s="66" t="s">
+      <c r="B54" s="66" t="s">
         <v>162</v>
       </c>
-      <c r="C53" s="67">
+      <c r="C54" s="67">
         <v>0.1</v>
       </c>
-      <c r="D53" s="20">
+      <c r="D54" s="20">
         <v>45594</v>
       </c>
-      <c r="E53" s="82">
+      <c r="E54" s="82">
         <v>4205277</v>
       </c>
-      <c r="F53" s="82"/>
-      <c r="G53" s="82"/>
-      <c r="H53" s="11" t="s">
+      <c r="F54" s="82"/>
+      <c r="G54" s="82"/>
+      <c r="H54" s="11" t="s">
         <v>38</v>
       </c>
     </row>
@@ -5799,7 +5836,7 @@
   <mergeCells count="8">
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A5:H5"/>

</xml_diff>